<commit_message>
Publish the rewritten Statistics, Microeconomics and Advanced teaching labs
The standalone teaching directory now matches private source 7242d518:
60 rewritten handouts and instructor companions with verified journal
cases, figures drawn with OpenEconometrics Charts, and corrected Advanced
Lab 12 and 20 dictionaries. Entry files keep the index.md layout and
PUBLICATION-MANIFEST.json records every file's source and hashes. The fixed
SDK source inventory is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/teaching/advanced-econometrics/labs/12-polynomial-centering/polynomial_centering.xlsx
+++ b/teaching/advanced-econometrics/labs/12-polynomial-centering/polynomial_centering.xlsx
@@ -3738,10 +3738,10 @@
         <x:v>x</x:v>
       </x:c>
       <x:c r="B3" s="8" t="str">
-        <x:v>Exposure or predictor X</x:v>
+        <x:v>Regressor entering the polynomial (raw, not centered)</x:v>
       </x:c>
       <x:c r="C3" s="8" t="str">
-        <x:v>centered units</x:v>
+        <x:v>X units</x:v>
       </x:c>
       <x:c r="D3" s="8" t="str">
         <x:v>No missing values.</x:v>

</xml_diff>